<commit_message>
Apply reviewed Standard Bank message corrections
</commit_message>
<xml_diff>
--- a/SD-E4 Message ID Mappings.xlsx
+++ b/SD-E4 Message ID Mappings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iconinformationsystems-my.sharepoint.com/personal/thileshnee_chinnasamy_iconis_co_za/Documents/Documents/SD Foreclosures Reporting/ABSA Write Back/SBSA Messages/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="779" documentId="8_{B05531C0-448F-4F90-BE87-3294BADDC224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46BCE0D2-2AEA-4B90-8215-399AC5AB765E}"/>
+  <xr:revisionPtr revIDLastSave="780" documentId="8_{B05531C0-448F-4F90-BE87-3294BADDC224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2120696-276A-43D8-8910-5C9454C92A0B}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-3285" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SD-E4 Message Mappings" sheetId="3" r:id="rId1"/>
@@ -695,7 +695,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -763,58 +763,37 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -833,10 +812,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1160,7 +1135,7 @@
     <col min="20" max="20" width="13.36328125" style="2" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="10.453125" style="2" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="5.08984375" style="28" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="5.08984375" style="2" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="8.453125" style="2" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="9.453125" style="2" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="8.90625" style="2" bestFit="1" customWidth="1"/>
@@ -1182,52 +1157,52 @@
     <col min="43" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:41" s="34" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="31" t="s">
+    <row r="2" spans="1:41" s="25" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A2" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="32"/>
-      <c r="P2" s="32"/>
-      <c r="Q2" s="32"/>
-      <c r="R2" s="32"/>
-      <c r="S2" s="32"/>
-      <c r="T2" s="32"/>
-      <c r="U2" s="32"/>
-      <c r="V2" s="32"/>
-      <c r="W2" s="33"/>
-      <c r="X2" s="32"/>
-      <c r="Y2" s="32"/>
-      <c r="Z2" s="32"/>
-      <c r="AA2" s="32"/>
-      <c r="AB2" s="32"/>
-      <c r="AC2" s="32"/>
-      <c r="AD2" s="32"/>
-      <c r="AE2" s="32"/>
-      <c r="AF2" s="32"/>
-      <c r="AG2" s="32"/>
-      <c r="AH2" s="32"/>
-      <c r="AI2" s="32"/>
-      <c r="AJ2" s="32"/>
-      <c r="AK2" s="32"/>
-      <c r="AL2" s="32"/>
-      <c r="AM2" s="32"/>
-      <c r="AN2" s="32"/>
-      <c r="AO2" s="32"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
+      <c r="L2" s="24"/>
+      <c r="M2" s="24"/>
+      <c r="N2" s="24"/>
+      <c r="O2" s="24"/>
+      <c r="P2" s="24"/>
+      <c r="Q2" s="24"/>
+      <c r="R2" s="24"/>
+      <c r="S2" s="24"/>
+      <c r="T2" s="24"/>
+      <c r="U2" s="24"/>
+      <c r="V2" s="24"/>
+      <c r="W2" s="24"/>
+      <c r="X2" s="24"/>
+      <c r="Y2" s="24"/>
+      <c r="Z2" s="24"/>
+      <c r="AA2" s="24"/>
+      <c r="AB2" s="24"/>
+      <c r="AC2" s="24"/>
+      <c r="AD2" s="24"/>
+      <c r="AE2" s="24"/>
+      <c r="AF2" s="24"/>
+      <c r="AG2" s="24"/>
+      <c r="AH2" s="24"/>
+      <c r="AI2" s="24"/>
+      <c r="AJ2" s="24"/>
+      <c r="AK2" s="24"/>
+      <c r="AL2" s="24"/>
+      <c r="AM2" s="24"/>
+      <c r="AN2" s="24"/>
+      <c r="AO2" s="24"/>
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.35">
       <c r="C3" s="22"/>
@@ -1250,7 +1225,7 @@
       <c r="T3" s="22"/>
       <c r="U3" s="22"/>
       <c r="V3" s="22"/>
-      <c r="W3" s="27"/>
+      <c r="W3" s="22"/>
       <c r="X3" s="22"/>
       <c r="Y3" s="22"/>
       <c r="Z3" s="22"/>
@@ -1277,23 +1252,23 @@
       <c r="B4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="E4" s="26" t="s">
+      <c r="E4" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A5" s="12"/>
       <c r="B5" s="12"/>
-      <c r="C5" s="36">
+      <c r="C5" s="27">
         <v>20121005</v>
       </c>
-      <c r="D5" s="40">
+      <c r="D5" s="31">
         <v>20121005161244</v>
       </c>
       <c r="E5" s="3"/>
@@ -1305,19 +1280,19 @@
       <c r="B7" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="26" t="s">
+      <c r="E7" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="F7" s="39" t="s">
+      <c r="F7" s="30" t="s">
         <v>160</v>
       </c>
-      <c r="G7" s="39" t="s">
+      <c r="G7" s="30" t="s">
         <v>162</v>
       </c>
       <c r="H7" s="3" t="s">
@@ -1328,30 +1303,30 @@
       <c r="A8" s="12"/>
       <c r="B8" s="12"/>
       <c r="C8" s="3"/>
-      <c r="D8" s="36">
+      <c r="D8" s="27">
         <v>20121005</v>
       </c>
-      <c r="E8" s="40">
+      <c r="E8" s="31">
         <v>20121005161244</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="G8" s="36">
+      <c r="G8" s="27">
         <v>20120701</v>
       </c>
-      <c r="H8" s="36" t="s">
+      <c r="H8" s="27" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:41" x14ac:dyDescent="0.35">
-      <c r="P9" s="35"/>
+      <c r="P9" s="26"/>
     </row>
     <row r="10" spans="1:41" ht="31" x14ac:dyDescent="0.35">
-      <c r="A10" s="24">
+      <c r="A10" s="33">
         <v>304</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="32" t="s">
         <v>12</v>
       </c>
       <c r="C10" s="13" t="s">
@@ -1360,7 +1335,7 @@
       <c r="D10" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="E10" s="26" t="s">
+      <c r="E10" s="6" t="s">
         <v>3</v>
       </c>
       <c r="F10" s="19" t="s">
@@ -1390,24 +1365,24 @@
       <c r="N10" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="O10" s="26" t="s">
+      <c r="O10" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="P10" s="35"/>
+      <c r="P10" s="26"/>
     </row>
     <row r="11" spans="1:41" x14ac:dyDescent="0.35">
-      <c r="A11" s="24"/>
-      <c r="B11" s="23"/>
-      <c r="C11" s="36">
+      <c r="A11" s="33"/>
+      <c r="B11" s="32"/>
+      <c r="C11" s="27">
         <v>1372</v>
       </c>
       <c r="D11" s="19" t="s">
         <v>166</v>
       </c>
-      <c r="E11" s="36">
+      <c r="E11" s="27">
         <v>20121030</v>
       </c>
-      <c r="F11" s="36">
+      <c r="F11" s="27">
         <v>20121113</v>
       </c>
       <c r="G11" s="6" t="s">
@@ -1427,7 +1402,7 @@
         <v>104</v>
       </c>
       <c r="O11" s="3"/>
-      <c r="P11" s="35"/>
+      <c r="P11" s="26"/>
     </row>
     <row r="12" spans="1:41" x14ac:dyDescent="0.35">
       <c r="B12" s="1"/>
@@ -1445,16 +1420,16 @@
       <c r="N12" s="8"/>
     </row>
     <row r="14" spans="1:41" ht="108.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="24">
+      <c r="A14" s="33">
         <v>321</v>
       </c>
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D14" s="26" t="s">
+      <c r="D14" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E14" s="6" t="s">
@@ -1517,24 +1492,24 @@
       <c r="X14" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="Y14" s="26" t="s">
+      <c r="Y14" s="6" t="s">
         <v>4</v>
       </c>
       <c r="Z14"/>
       <c r="AA14"/>
     </row>
     <row r="15" spans="1:41" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="24"/>
-      <c r="B15" s="23"/>
+      <c r="A15" s="33"/>
+      <c r="B15" s="32"/>
       <c r="C15" s="6"/>
       <c r="D15" s="7"/>
       <c r="E15" s="6">
         <v>1235</v>
       </c>
-      <c r="F15" s="36">
+      <c r="F15" s="27">
         <v>20150805</v>
       </c>
-      <c r="G15" s="36" t="s">
+      <c r="G15" s="27" t="s">
         <v>167</v>
       </c>
       <c r="H15" s="7"/>
@@ -1596,7 +1571,7 @@
       <c r="T16" s="9"/>
       <c r="U16" s="8"/>
       <c r="V16" s="8"/>
-      <c r="W16" s="29"/>
+      <c r="W16" s="8"/>
       <c r="X16" s="8"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.35">
@@ -1609,7 +1584,7 @@
       <c r="C18" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D18" s="26" t="s">
+      <c r="D18" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E18" s="6" t="s">
@@ -1621,10 +1596,10 @@
       <c r="G18" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="H18" s="26" t="s">
+      <c r="H18" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="I18" s="35"/>
+      <c r="I18" s="26"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B19" s="1"/>
@@ -1644,10 +1619,10 @@
       <c r="C21" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D21" s="26" t="s">
+      <c r="D21" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="E21" s="26" t="s">
+      <c r="E21" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1664,7 +1639,7 @@
       <c r="C24" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D24" s="26" t="s">
+      <c r="D24" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E24" s="3" t="s">
@@ -1673,7 +1648,7 @@
       <c r="F24" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="G24" s="26" t="s">
+      <c r="G24" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1681,11 +1656,11 @@
       <c r="A25" s="12"/>
       <c r="B25" s="12"/>
       <c r="C25" s="3"/>
-      <c r="D25" s="37"/>
-      <c r="E25" s="37" t="s">
+      <c r="D25" s="28"/>
+      <c r="E25" s="28" t="s">
         <v>158</v>
       </c>
-      <c r="F25" s="37" t="s">
+      <c r="F25" s="28" t="s">
         <v>158</v>
       </c>
       <c r="G25" s="3"/>
@@ -1700,7 +1675,7 @@
       <c r="C28" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D28" s="26" t="s">
+      <c r="D28" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E28" s="6" t="s">
@@ -1715,7 +1690,7 @@
       <c r="H28" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="I28" s="26" t="s">
+      <c r="I28" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1749,7 +1724,7 @@
       <c r="C32" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D32" s="26" t="s">
+      <c r="D32" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E32" s="6" t="s">
@@ -1782,20 +1757,20 @@
       <c r="N32" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="O32" s="26" t="s">
+      <c r="O32" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="P32" s="35"/>
+      <c r="P32" s="26"/>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A33" s="12"/>
       <c r="B33" s="4"/>
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
-      <c r="E33" s="37" t="s">
+      <c r="E33" s="28" t="s">
         <v>171</v>
       </c>
-      <c r="F33" s="37" t="s">
+      <c r="F33" s="28" t="s">
         <v>170</v>
       </c>
       <c r="G33" s="6" t="s">
@@ -1809,7 +1784,7 @@
       <c r="M33" s="6"/>
       <c r="N33" s="7"/>
       <c r="O33" s="3"/>
-      <c r="P33" s="35"/>
+      <c r="P33" s="26"/>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B34" s="18"/>
@@ -1837,7 +1812,7 @@
       <c r="C36" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D36" s="26" t="s">
+      <c r="D36" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E36" s="6" t="s">
@@ -1846,7 +1821,7 @@
       <c r="F36" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="G36" s="26" t="s">
+      <c r="G36" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1855,10 +1830,10 @@
       <c r="B37" s="12"/>
       <c r="C37" s="6"/>
       <c r="D37" s="3"/>
-      <c r="E37" s="37" t="s">
+      <c r="E37" s="28" t="s">
         <v>171</v>
       </c>
-      <c r="F37" s="37" t="s">
+      <c r="F37" s="28" t="s">
         <v>170</v>
       </c>
       <c r="G37" s="3"/>
@@ -1878,13 +1853,13 @@
       <c r="C40" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D40" s="26" t="s">
+      <c r="D40" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="F40" s="26" t="s">
+      <c r="F40" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1893,7 +1868,7 @@
       <c r="B41" s="12"/>
       <c r="C41" s="6"/>
       <c r="D41" s="3"/>
-      <c r="E41" s="37" t="s">
+      <c r="E41" s="28" t="s">
         <v>169</v>
       </c>
       <c r="F41" s="3"/>
@@ -1912,7 +1887,7 @@
       <c r="C44" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D44" s="26" t="s">
+      <c r="D44" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E44" s="6" t="s">
@@ -1921,10 +1896,10 @@
       <c r="F44" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="G44" s="38" t="s">
+      <c r="G44" s="29" t="s">
         <v>173</v>
       </c>
-      <c r="H44" s="26" t="s">
+      <c r="H44" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1952,13 +1927,13 @@
       <c r="C47" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D47" s="26" t="s">
+      <c r="D47" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="F47" s="26" t="s">
+      <c r="F47" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1974,7 +1949,7 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="12">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B50" s="12" t="s">
         <v>57</v>
@@ -1982,7 +1957,7 @@
       <c r="C50" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D50" s="26" t="s">
+      <c r="D50" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E50" s="6" t="s">
@@ -1991,7 +1966,7 @@
       <c r="F50" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G50" s="26" t="s">
+      <c r="G50" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2018,7 +1993,7 @@
       <c r="C54" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D54" s="26" t="s">
+      <c r="D54" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E54" s="6" t="s">
@@ -2027,7 +2002,7 @@
       <c r="F54" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="G54" s="26" t="s">
+      <c r="G54" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2039,7 +2014,7 @@
       <c r="E55" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="F55" s="36" t="s">
+      <c r="F55" s="27" t="s">
         <v>174</v>
       </c>
       <c r="G55" s="3"/>
@@ -2054,7 +2029,7 @@
       <c r="C57" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D57" s="26" t="s">
+      <c r="D57" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E57" s="3" t="s">
@@ -2066,7 +2041,7 @@
       <c r="G57" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="H57" s="26" t="s">
+      <c r="H57" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2096,7 +2071,7 @@
       <c r="C61" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D61" s="26" t="s">
+      <c r="D61" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E61" s="3" t="s">
@@ -2105,7 +2080,7 @@
       <c r="F61" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="G61" s="26" t="s">
+      <c r="G61" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2192,7 +2167,7 @@
       <c r="W65" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="X65" s="26" t="s">
+      <c r="X65" s="6" t="s">
         <v>159</v>
       </c>
       <c r="Y65" s="19" t="s">
@@ -2246,7 +2221,7 @@
       <c r="AO65" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="AP65" s="26" t="s">
+      <c r="AP65" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2283,7 +2258,7 @@
       <c r="T66" s="6"/>
       <c r="U66" s="6"/>
       <c r="V66" s="6"/>
-      <c r="W66" s="26"/>
+      <c r="W66" s="6"/>
       <c r="X66" s="6"/>
       <c r="Y66" s="6" t="s">
         <v>104</v>
@@ -2339,7 +2314,7 @@
       <c r="T67" s="8"/>
       <c r="U67" s="8"/>
       <c r="V67" s="8"/>
-      <c r="W67" s="29"/>
+      <c r="W67" s="8"/>
       <c r="X67" s="8"/>
       <c r="Y67" s="9"/>
       <c r="Z67" s="8"/>
@@ -2368,7 +2343,7 @@
       <c r="C69" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D69" s="26" t="s">
+      <c r="D69" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E69" s="6" t="s">
@@ -2383,7 +2358,7 @@
       <c r="H69" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="I69" s="26" t="s">
+      <c r="I69" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2395,13 +2370,13 @@
       <c r="E70" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="F70" s="36" t="s">
+      <c r="F70" s="27" t="s">
         <v>175</v>
       </c>
-      <c r="G70" s="36">
+      <c r="G70" s="27">
         <v>20141010</v>
       </c>
-      <c r="H70" s="36">
+      <c r="H70" s="27">
         <v>20191011</v>
       </c>
       <c r="I70" s="3"/>
@@ -2416,7 +2391,7 @@
       <c r="C72" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D72" s="26" t="s">
+      <c r="D72" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E72" s="21" t="s">
@@ -2428,7 +2403,7 @@
       <c r="G72" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="H72" s="26" t="s">
+      <c r="H72" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2454,7 +2429,7 @@
       <c r="C76" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D76" s="26" t="s">
+      <c r="D76" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E76" s="6" t="s">
@@ -2469,7 +2444,7 @@
       <c r="H76" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="I76" s="26" t="s">
+      <c r="I76" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2498,7 +2473,7 @@
       <c r="C80" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D80" s="26" t="s">
+      <c r="D80" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E80" s="6" t="s">
@@ -2546,11 +2521,11 @@
       <c r="S80" s="19" t="s">
         <v>137</v>
       </c>
-      <c r="T80" s="26" t="s">
+      <c r="T80" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="81" spans="1:23" s="11" customFormat="1" ht="46.5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:20" s="11" customFormat="1" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A81" s="5"/>
       <c r="B81" s="5"/>
       <c r="C81" s="7">
@@ -2603,9 +2578,8 @@
         <v>142</v>
       </c>
       <c r="T81" s="3"/>
-      <c r="W81" s="30"/>
-    </row>
-    <row r="82" spans="1:23" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="82" spans="1:20" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
       <c r="C82" s="9"/>
@@ -2620,9 +2594,8 @@
       <c r="P82" s="8"/>
       <c r="Q82" s="16"/>
       <c r="R82" s="16"/>
-      <c r="W82" s="30"/>
-    </row>
-    <row r="84" spans="1:23" ht="31" x14ac:dyDescent="0.35">
+    </row>
+    <row r="84" spans="1:20" ht="31" x14ac:dyDescent="0.35">
       <c r="A84" s="12">
         <v>421</v>
       </c>
@@ -2632,7 +2605,7 @@
       <c r="C84" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D84" s="26" t="s">
+      <c r="D84" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E84" s="3" t="s">
@@ -2647,14 +2620,14 @@
       <c r="H84" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="I84" s="26" t="s">
+      <c r="I84" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="85" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.35">
       <c r="C85" s="8"/>
     </row>
-    <row r="87" spans="1:23" ht="31" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:20" ht="31" x14ac:dyDescent="0.35">
       <c r="A87" s="12">
         <v>428</v>
       </c>
@@ -2679,11 +2652,11 @@
       <c r="H87" s="20" t="s">
         <v>153</v>
       </c>
-      <c r="I87" s="26" t="s">
+      <c r="I87" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="88" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A88" s="12"/>
       <c r="B88" s="12"/>
       <c r="C88" s="6"/>
@@ -2700,7 +2673,7 @@
       </c>
       <c r="I88" s="3"/>
     </row>
-    <row r="90" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A90" s="12">
         <v>430</v>
       </c>
@@ -2710,7 +2683,7 @@
       <c r="C90" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D90" s="26" t="s">
+      <c r="D90" s="6" t="s">
         <v>159</v>
       </c>
       <c r="E90" s="13" t="s">
@@ -2719,11 +2692,11 @@
       <c r="F90" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="G90" s="26" t="s">
+      <c r="G90" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="91" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A91" s="12"/>
       <c r="B91" s="12"/>
       <c r="C91" s="3"/>

</xml_diff>